<commit_message>
announcement end to end
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0E879495-1495-4649-85E3-79B64AC23CFF}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{83774BC0-5AA3-4EC8-8A03-E621DC4DAD64}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" activeTab="2" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Edition" sheetId="2" r:id="rId2"/>
     <sheet name="BudgetPeriod" sheetId="3" r:id="rId3"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="53">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -162,6 +163,30 @@
   </si>
   <si>
     <t>BudgetEndDate__c</t>
+  </si>
+  <si>
+    <t>ReviewerRole__c</t>
+  </si>
+  <si>
+    <t>Fiscal Reviewer</t>
+  </si>
+  <si>
+    <t>Name__c</t>
+  </si>
+  <si>
+    <t>Automation FO</t>
+  </si>
+  <si>
+    <t>Review Financial details</t>
+  </si>
+  <si>
+    <t>DueDate__c</t>
+  </si>
+  <si>
+    <t>Responsibility__c</t>
+  </si>
+  <si>
+    <t>TextArea</t>
   </si>
 </sst>
 </file>
@@ -956,4 +981,88 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.36328125" customWidth="1"/>
+    <col min="3" max="4" width="20.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated all the feature files to be independent
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{7AC67643-9CF8-4D4D-9D40-8BB3BCC90E2F}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{4AA1649A-E379-48EB-94F0-C01CF75A4F49}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -49,9 +49,6 @@
     <t>Text</t>
   </si>
   <si>
-    <t>Automation Announcement</t>
-  </si>
-  <si>
     <t>Dropdown</t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>RiskAssessment_Required__c</t>
+  </si>
+  <si>
+    <t>Automation Announcement to be deleted</t>
   </si>
 </sst>
 </file>
@@ -568,7 +568,7 @@
     <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -593,10 +593,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -604,13 +604,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -618,13 +618,13 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -632,13 +632,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -674,83 +674,83 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D7">
         <v>10</v>
@@ -758,41 +758,41 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
         <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
         <v>25</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -800,13 +800,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
         <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
       </c>
       <c r="D11">
         <v>10</v>
@@ -814,27 +814,27 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -842,13 +842,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D14">
         <v>5</v>
@@ -856,27 +856,27 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D16">
         <v>1000</v>
@@ -884,13 +884,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17">
         <v>10000</v>
@@ -898,13 +898,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -912,13 +912,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s">
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19">
         <v>100000</v>
@@ -962,10 +962,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2">
         <v>15</v>
@@ -976,10 +976,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3">
         <v>379</v>
@@ -1018,13 +1018,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
         <v>45</v>
-      </c>
-      <c r="D2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1032,13 +1032,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
         <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1046,13 +1046,13 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1060,10 +1060,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1081,13 +1081,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D1">
         <v>8</v>

</xml_diff>

<commit_message>
All changes done to feature files so that each test case is independent of the other
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{4AA1649A-E379-48EB-94F0-C01CF75A4F49}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0DF50632-8499-422A-BBDB-17AC648FE97C}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -568,7 +568,7 @@
     <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.453125" customWidth="1"/>
+    <col min="4" max="4" width="43.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
All script working until application review
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0DF50632-8499-422A-BBDB-17AC648FE97C}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{BFD365EA-EC3C-40E6-8F56-029932DF3D06}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6960" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Reviewer" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="179017"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -58,9 +58,6 @@
     <t>AnnouncementType__c</t>
   </si>
   <si>
-    <t>Competitive</t>
-  </si>
-  <si>
     <t>Lookup</t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>Automation Announcement to be deleted</t>
+  </si>
+  <si>
+    <t>Directed</t>
   </si>
 </sst>
 </file>
@@ -562,16 +562,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,7 +585,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -596,49 +596,35 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
         <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -650,15 +636,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -672,253 +658,253 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
         <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
       </c>
       <c r="D11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D16">
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17">
         <v>10000</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D18">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D19">
         <v>100000</v>
@@ -935,15 +921,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -957,29 +943,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D2">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D3">
         <v>379</v>
@@ -993,13 +979,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.36328125" customWidth="1"/>
-    <col min="3" max="4" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1021,49 +1008,49 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" t="s">
         <v>44</v>
       </c>
-      <c r="D2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
         <v>46</v>
       </c>
-      <c r="D3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1076,21 +1063,35 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D1">
         <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated common steps in feature file to match with Utah common steps and created two Site visit Test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{BFD365EA-EC3C-40E6-8F56-029932DF3D06}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{640A57A5-E109-4FE4-AC98-BA0F821F1DDC}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -64,9 +64,6 @@
     <t>Program__c</t>
   </si>
   <si>
-    <t>Automation Program</t>
-  </si>
-  <si>
     <t>Budget_Category_Package__c</t>
   </si>
   <si>
@@ -190,10 +187,13 @@
     <t>RiskAssessment_Required__c</t>
   </si>
   <si>
-    <t>Automation Announcement to be deleted</t>
-  </si>
-  <si>
     <t>Directed</t>
+  </si>
+  <si>
+    <t>Automation Announcement Dec10</t>
+  </si>
+  <si>
+    <t>PG--0245</t>
   </si>
 </sst>
 </file>
@@ -563,15 +563,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,7 +585,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -599,7 +599,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -609,11 +609,11 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -621,30 +621,33 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" tooltip="PG--0245" display="https://test7-internal--c.na57.visual.force.com/a3b0b000001dxL3AAI" xr:uid="{16111789-5187-4372-A131-EB21311CAC9C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -658,253 +661,253 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
       </c>
       <c r="D11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16">
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D17">
         <v>10000</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D18">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D19">
         <v>100000</v>
@@ -921,15 +924,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -943,29 +946,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D2">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3">
         <v>379</v>
@@ -979,14 +982,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1000,7 +1003,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1008,13 +1011,13 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>43</v>
       </c>
-      <c r="D2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1022,35 +1025,35 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="D3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1064,23 +1067,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D1">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1091,7 +1094,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified the consolidated methods for announcement and application intake feature
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{640A57A5-E109-4FE4-AC98-BA0F821F1DDC}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{F7DFDDE1-C591-4C55-AEE5-6DF36E5DC62A}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -100,9 +100,6 @@
     <t>MultiSelect</t>
   </si>
   <si>
-    <t>["State governments", "Independent school districts"]</t>
-  </si>
-  <si>
     <t>ReleaseDate__c</t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>PG--0245</t>
+  </si>
+  <si>
+    <t>State governments;Independent school districts</t>
   </si>
 </sst>
 </file>
@@ -562,74 +562,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" tooltip="PG--0245" display="https://test7-internal--c.na57.visual.force.com/a3b0b000001dxL3AAI" xr:uid="{16111789-5187-4372-A131-EB21311CAC9C}"/>
+    <hyperlink ref="C3" r:id="rId1" tooltip="PG--0245" display="https://test7-internal--c.na57.visual.force.com/a3b0b000001dxL3AAI" xr:uid="{16111789-5187-4372-A131-EB21311CAC9C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId2"/>
@@ -638,284 +625,226 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
         <v>26</v>
       </c>
-      <c r="D11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
       <c r="C12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13">
+      <c r="C17">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
         <v>29</v>
       </c>
-      <c r="B16" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19">
+      <c r="C19">
         <v>100000</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D15" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
+    <hyperlink ref="C15" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -923,54 +852,44 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2">
+        <v>39</v>
+      </c>
+      <c r="C2">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3">
+        <v>40</v>
+      </c>
+      <c r="C3">
         <v>379</v>
       </c>
     </row>
@@ -981,81 +900,65 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
         <v>44</v>
       </c>
-      <c r="D3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5">
+        <v>46</v>
+      </c>
+      <c r="C5">
         <v>3</v>
       </c>
     </row>
@@ -1066,24 +969,70 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D1">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1094,7 +1043,94 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the consolidated methods and steps in Application Review
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{F7DFDDE1-C591-4C55-AEE5-6DF36E5DC62A}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{6F537260-6439-41D9-9D41-E56DEB7FE369}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -187,13 +187,13 @@
     <t>Directed</t>
   </si>
   <si>
-    <t>Automation Announcement Dec10</t>
-  </si>
-  <si>
-    <t>PG--0245</t>
-  </si>
-  <si>
     <t>State governments;Independent school districts</t>
+  </si>
+  <si>
+    <t>Automation Announcement Dec25</t>
+  </si>
+  <si>
+    <t>PG--0271</t>
   </si>
 </sst>
 </file>
@@ -589,7 +589,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -599,8 +599,8 @@
       <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>53</v>
+      <c r="C3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -615,11 +615,8 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" tooltip="PG--0245" display="https://test7-internal--c.na57.visual.force.com/a3b0b000001dxL3AAI" xr:uid="{16111789-5187-4372-A131-EB21311CAC9C}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId2"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -729,7 +726,7 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
All Payment Request Test Cases are done
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{6F537260-6439-41D9-9D41-E56DEB7FE369}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0A44CA38-1B3B-42EC-B315-973353A7AD9F}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="57">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -190,10 +190,16 @@
     <t>State governments;Independent school districts</t>
   </si>
   <si>
-    <t>Automation Announcement Dec25</t>
-  </si>
-  <si>
-    <t>PG--0271</t>
+    <t>Automation Announcement Jan10</t>
+  </si>
+  <si>
+    <t>PG--0294</t>
+  </si>
+  <si>
+    <t>WBSRequired__c</t>
+  </si>
+  <si>
+    <t>AreExpensesBuildIUpLevel__c</t>
   </si>
 </sst>
 </file>
@@ -563,14 +569,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -581,7 +587,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -592,7 +598,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -603,7 +609,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -622,15 +628,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -641,7 +647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -652,196 +658,207 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>50</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>33</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
         <v>34</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C17">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>28</v>
       </c>
       <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" t="s">
         <v>29</v>
       </c>
-      <c r="C19">
+      <c r="C20">
         <v>100000</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C15" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
+    <hyperlink ref="C16" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -850,14 +867,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -868,7 +885,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -879,7 +896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -898,13 +915,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -915,7 +932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -926,7 +943,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -937,7 +954,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -948,7 +965,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -966,16 +983,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
-  <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1001,7 +1018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G2" t="s">
         <v>5</v>
       </c>
@@ -1015,7 +1032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G3" t="s">
         <v>9</v>
       </c>
@@ -1029,7 +1046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1052,7 +1069,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H5" t="s">
         <v>6</v>
       </c>
@@ -1060,74 +1077,85 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H19" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Progress report test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0A44CA38-1B3B-42EC-B315-973353A7AD9F}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8820B2CF-A3E7-4CC4-BADF-915BB79EB9F2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -190,16 +190,16 @@
     <t>State governments;Independent school districts</t>
   </si>
   <si>
-    <t>Automation Announcement Jan10</t>
-  </si>
-  <si>
-    <t>PG--0294</t>
-  </si>
-  <si>
     <t>WBSRequired__c</t>
   </si>
   <si>
     <t>AreExpensesBuildIUpLevel__c</t>
+  </si>
+  <si>
+    <t>PG--0303</t>
+  </si>
+  <si>
+    <t>Automation Announcement FOR Jan16</t>
   </si>
 </sst>
 </file>
@@ -569,14 +569,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,7 +587,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -595,10 +595,10 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -606,10 +606,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -629,14 +629,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -647,7 +647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -658,7 +658,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -669,7 +669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -680,7 +680,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -691,7 +691,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -702,18 +702,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -724,18 +724,18 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -746,7 +746,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -757,7 +757,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -768,7 +768,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -779,7 +779,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -790,7 +790,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -801,7 +801,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -812,7 +812,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -823,7 +823,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -834,7 +834,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -845,7 +845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -867,14 +867,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -885,7 +885,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -896,7 +896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -915,13 +915,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -932,7 +932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -943,7 +943,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -954,7 +954,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -965,7 +965,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -984,15 +984,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G2" t="s">
         <v>5</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G3" t="s">
         <v>9</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H5" t="s">
         <v>6</v>
       </c>
@@ -1077,77 +1077,77 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
updated the old test cases in program announcement
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C04D10-4CC7-4E8E-A9A1-EC0F36C17E1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1997D956-2B98-4A80-9CEA-F15CFBC57BCE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -199,7 +199,7 @@
     <t>PG--0314</t>
   </si>
   <si>
-    <t>Automation Announcement Jan18</t>
+    <t>Automation Announcement Jan18 -1</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
selectboxes method xpath is updated
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1997D956-2B98-4A80-9CEA-F15CFBC57BCE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA74A5AF-E2C2-4878-8061-C967F539DFF8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -196,10 +196,10 @@
     <t>AreExpensesBuildIUpLevel__c</t>
   </si>
   <si>
-    <t>PG--0314</t>
-  </si>
-  <si>
-    <t>Automation Announcement Jan18 -1</t>
+    <t>PG--0342</t>
+  </si>
+  <si>
+    <t>Automation Announcement Jan19</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
All test cases until application review is working
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA74A5AF-E2C2-4878-8061-C967F539DFF8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74C062C3-5D8E-437B-BD23-6EB33E2C5F92}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -196,10 +196,10 @@
     <t>AreExpensesBuildIUpLevel__c</t>
   </si>
   <si>
-    <t>PG--0342</t>
-  </si>
-  <si>
-    <t>Automation Announcement Jan19</t>
+    <t>Automation Announcement Jan19 Vi</t>
+  </si>
+  <si>
+    <t>PG--0343</t>
   </si>
 </sst>
 </file>
@@ -595,7 +595,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,7 +606,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Removed the ProtalType method
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D989430-3484-4BD9-B554-FA25B6ED798B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46345F1F-2A50-4BA0-AFED-8B2310B5BDDD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -199,7 +199,7 @@
     <t>PG--0370</t>
   </si>
   <si>
-    <t>Automation Announcement Jan25</t>
+    <t>Automation Announcement Regression</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Announcement creation step updated
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22DED1F8-0A0F-4DD3-AD42-E904DD8AE6E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA8BC59-B047-4515-87BF-B5CFEC3C3611}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Edition" sheetId="2" r:id="rId2"/>
     <sheet name="BudgetPeriod" sheetId="3" r:id="rId3"/>
     <sheet name="Reviewer" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="62">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -196,10 +197,25 @@
     <t>AreExpensesBuildIUpLevel__c</t>
   </si>
   <si>
-    <t>Automation Announcement Jan5</t>
-  </si>
-  <si>
     <t>PG-TAO-0011</t>
+  </si>
+  <si>
+    <t>FocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>IsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>KPIsRequired__c</t>
+  </si>
+  <si>
+    <t>IsAdvancePermitted__c</t>
+  </si>
+  <si>
+    <t>IsNegotiationsAllowed__c</t>
+  </si>
+  <si>
+    <t>Automation Announcement Regression</t>
   </si>
 </sst>
 </file>
@@ -595,7 +611,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,7 +622,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -628,7 +644,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -652,10 +668,10 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -663,10 +679,10 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -674,10 +690,10 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>30</v>
+        <v>25</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -685,7 +701,7 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
         <v>30</v>
@@ -696,10 +712,10 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>49</v>
+        <v>33</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -707,10 +723,10 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" t="s">
-        <v>49</v>
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -718,147 +734,59 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" t="s">
-        <v>49</v>
+        <v>37</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>52</v>
+        <v>38</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C12">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20">
         <v>100000</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C16" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
+    <hyperlink ref="C8" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -982,6 +910,175 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
updated the announcement feature file
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA8BC59-B047-4515-87BF-B5CFEC3C3611}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9631D516-A63D-40FF-BAEC-4013DF9EAA08}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -215,7 +215,7 @@
     <t>IsNegotiationsAllowed__c</t>
   </si>
   <si>
-    <t>Automation Announcement Regression</t>
+    <t>Automation Announcement Feb15</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fixing the test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9631D516-A63D-40FF-BAEC-4013DF9EAA08}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEA09DD-BDE9-4C12-BAEF-F9FFEF34E003}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7332" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -197,9 +197,6 @@
     <t>AreExpensesBuildIUpLevel__c</t>
   </si>
   <si>
-    <t>PG-TAO-0011</t>
-  </si>
-  <si>
     <t>FocusAreaRequired__c</t>
   </si>
   <si>
@@ -215,7 +212,10 @@
     <t>IsNegotiationsAllowed__c</t>
   </si>
   <si>
-    <t>Automation Announcement Feb15</t>
+    <t>PG-TAO-0055</t>
+  </si>
+  <si>
+    <t>Automation Announcement Regression</t>
   </si>
 </sst>
 </file>
@@ -585,14 +585,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -603,7 +603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -614,7 +614,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -622,10 +622,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -645,14 +645,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -663,7 +663,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -674,7 +674,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -685,7 +685,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -696,7 +696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -707,7 +707,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -718,7 +718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -729,7 +729,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -740,7 +740,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -751,7 +751,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -762,7 +762,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -795,14 +795,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -813,7 +813,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -824,7 +824,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -843,13 +843,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -860,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -871,7 +871,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -882,7 +882,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -893,7 +893,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -912,13 +912,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -929,7 +929,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -940,7 +940,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -951,7 +951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -962,7 +962,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -973,7 +973,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -984,7 +984,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -995,7 +995,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1006,40 +1006,40 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1050,23 +1050,23 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
         <v>49</v>
@@ -1081,15 +1081,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G2" t="s">
         <v>5</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G3" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H5" t="s">
         <v>6</v>
       </c>
@@ -1174,77 +1174,77 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
updated the failing test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEA09DD-BDE9-4C12-BAEF-F9FFEF34E003}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3C33AE-5CDA-4151-A2FF-5C7749983442}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -212,10 +212,10 @@
     <t>IsNegotiationsAllowed__c</t>
   </si>
   <si>
-    <t>PG-TAO-0055</t>
-  </si>
-  <si>
-    <t>Automation Announcement Regression</t>
+    <t>PG-TAO-0063</t>
+  </si>
+  <si>
+    <t>Automation Announcement Feb21</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated the test scripts
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3C33AE-5CDA-4151-A2FF-5C7749983442}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E57EC4-B756-43E6-9FD5-D2E32D2038CA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
updated to project in excel
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E57EC4-B756-43E6-9FD5-D2E32D2038CA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494118F7-BFEA-441A-9B79-F00980A45D72}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7335" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -215,7 +215,7 @@
     <t>PG-TAO-0063</t>
   </si>
   <si>
-    <t>Automation Announcement Feb21</t>
+    <t>Automation Announcement</t>
   </si>
 </sst>
 </file>
@@ -585,14 +585,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -603,7 +603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -614,7 +614,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -625,7 +625,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -645,14 +645,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -663,7 +663,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -674,7 +674,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -685,7 +685,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -696,7 +696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -707,7 +707,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -718,7 +718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -729,7 +729,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -740,7 +740,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -751,7 +751,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -762,7 +762,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -795,14 +795,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -813,7 +813,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -824,7 +824,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -843,13 +843,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -860,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -871,7 +871,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -882,7 +882,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -893,7 +893,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -912,13 +912,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -929,7 +929,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -940,7 +940,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -951,7 +951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -962,7 +962,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -973,7 +973,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -984,7 +984,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -995,7 +995,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1081,15 +1081,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G2" t="s">
         <v>5</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G3" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H5" t="s">
         <v>6</v>
       </c>
@@ -1174,77 +1174,77 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2038: Merge applicationintake-refactoring to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FA4139-B1C6-4E98-8EED-FC6F39A45E2C}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E427883E-F532-4740-AD35-7E7C826298A7}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -179,18 +179,6 @@
     <t>AllowRecordEdit__c</t>
   </si>
   <si>
-    <t>Competitive Announcement for Automation</t>
-  </si>
-  <si>
-    <t>Directed Announcement for Automation</t>
-  </si>
-  <si>
-    <t>Formula Announcement for Automation</t>
-  </si>
-  <si>
-    <t>PG-TAO-0148</t>
-  </si>
-  <si>
     <t>Rating__c</t>
   </si>
   <si>
@@ -201,13 +189,25 @@
   </si>
   <si>
     <t>Reviewed</t>
+  </si>
+  <si>
+    <t>Automation Permanent Internal Program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Directed Announcement </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Competitive Announcement </t>
+  </si>
+  <si>
+    <t>Automation Formula Announcement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +219,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -245,7 +252,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -254,6 +261,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -596,7 +604,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,8 +614,8 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>51</v>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -656,7 +664,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -666,8 +674,8 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>51</v>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -715,7 +723,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -725,8 +733,8 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>51</v>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -774,7 +782,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -784,8 +792,8 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>51</v>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1267,10 +1275,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1278,10 +1286,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2102: Merge applicationintake-refactoring to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E427883E-F532-4740-AD35-7E7C826298A7}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4831A7F8-0D4E-4214-93F0-069962A5835C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="6" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="57">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>Automation Formula Announcement</t>
+  </si>
+  <si>
+    <t>DueDate__c</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1016,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
@@ -1036,10 +1039,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1047,10 +1050,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1069,9 +1072,20 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged PR 2174: Merge MahadevProduct2May to master
Done changes as per QA org, removed blank spaces from folder names under project
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4831A7F8-0D4E-4214-93F0-069962A5835C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484D7A8D-0692-407C-BAE2-3128426608ED}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="6" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="4" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -204,6 +204,12 @@
   </si>
   <si>
     <t>DueDate__c</t>
+  </si>
+  <si>
+    <t>fieldMaxApplicationsAllowed__c</t>
+  </si>
+  <si>
+    <t>100</t>
   </si>
 </sst>
 </file>
@@ -581,14 +587,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -599,7 +605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -610,7 +616,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -621,7 +627,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -641,14 +647,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,7 +665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -670,7 +676,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -681,7 +687,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -700,14 +706,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -718,7 +724,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -729,7 +735,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -740,7 +746,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -759,14 +765,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -777,7 +783,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -788,7 +794,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -799,7 +805,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -818,165 +824,177 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C10">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
       <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="C12">
+      <c r="C13">
         <v>100000</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C8" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -987,7 +1005,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -998,7 +1016,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1017,13 +1035,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1034,7 +1052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1045,7 +1063,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1056,7 +1074,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1067,7 +1085,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1078,7 +1096,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1098,13 +1116,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1115,7 +1133,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1126,7 +1144,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1137,7 +1155,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1148,7 +1166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1159,7 +1177,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1170,7 +1188,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1181,7 +1199,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1192,7 +1210,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1203,7 +1221,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1214,7 +1232,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1225,7 +1243,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1236,7 +1254,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1247,7 +1265,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1267,13 +1285,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1284,7 +1302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1295,7 +1313,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2175: Merge applicationintake-refactoring to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484D7A8D-0692-407C-BAE2-3128426608ED}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F4D287-E209-4028-8C2C-E0F27298675F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="4" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="12" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,14 @@
     <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId3"/>
     <sheet name="Creation" sheetId="7" r:id="rId4"/>
     <sheet name="Edition" sheetId="2" r:id="rId5"/>
-    <sheet name="BudgetPeriod" sheetId="3" r:id="rId6"/>
-    <sheet name="Reviewer" sheetId="4" r:id="rId7"/>
-    <sheet name="Creation Second Modal" sheetId="6" r:id="rId8"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId9"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId6"/>
+    <sheet name="BudgetPeriod" sheetId="3" r:id="rId7"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId8"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId9"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId10"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId11"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId12"/>
+    <sheet name="Sheet3" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -33,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -206,10 +210,10 @@
     <t>DueDate__c</t>
   </si>
   <si>
-    <t>fieldMaxApplicationsAllowed__c</t>
-  </si>
-  <si>
-    <t>100</t>
+    <t>MaxApplicationsAllowed__c</t>
+  </si>
+  <si>
+    <t>Automation Competitive Announcement for pre-application</t>
   </si>
 </sst>
 </file>
@@ -587,14 +591,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -605,7 +609,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -616,7 +620,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -627,7 +631,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -644,17 +648,453 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13">
+        <v>100000</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{E83D9309-0130-4FAC-B722-10EDB4BC1AA9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -665,7 +1105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -676,7 +1116,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -687,7 +1127,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -706,14 +1146,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -724,7 +1164,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -735,7 +1175,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -746,7 +1186,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -765,14 +1205,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -783,7 +1223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -794,7 +1234,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -805,7 +1245,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -824,177 +1264,314 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C10">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C11">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13">
         <v>100000</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C9" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
+    <hyperlink ref="C8" r:id="rId1" xr:uid="{E81D0B52-59DF-468B-AEC9-C98BD1BE50E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>100000</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1" xr:uid="{7A99DF26-2B2C-4867-910D-ECFCB9195B76}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1005,7 +1582,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1016,7 +1593,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1032,16 +1609,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1052,7 +1629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1063,7 +1640,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1074,7 +1651,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1085,7 +1662,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1096,7 +1673,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1113,16 +1690,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1133,7 +1710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1144,7 +1721,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1155,7 +1732,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1166,7 +1743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1177,7 +1754,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1188,7 +1765,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1199,7 +1776,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1210,7 +1787,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1221,7 +1798,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1232,7 +1809,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1243,7 +1820,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1254,7 +1831,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1265,7 +1842,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1280,52 +1857,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2229: Merge applicationintake-refactoring to master
updated Home Module
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F4D287-E209-4028-8C2C-E0F27298675F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B551A9-029B-42A6-B5F3-08103B0F05F0}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="12" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8964" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Merged PR 2419: Merge planningmodulenewscenarios to master
Related work items: #53285
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B551A9-029B-42A6-B5F3-08103B0F05F0}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA8ACBE-5ECE-44BA-891F-723783545872}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8964" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -22,10 +22,11 @@
     <sheet name="BudgetPeriod" sheetId="3" r:id="rId7"/>
     <sheet name="Reviewer" sheetId="4" r:id="rId8"/>
     <sheet name="Creation Second Modal" sheetId="6" r:id="rId9"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId10"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId11"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId12"/>
-    <sheet name="Sheet3" sheetId="13" r:id="rId13"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId10"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId11"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId12"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId13"/>
+    <sheet name="Sheet3" sheetId="13" r:id="rId14"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -201,9 +202,6 @@
     <t xml:space="preserve">Automation Directed Announcement </t>
   </si>
   <si>
-    <t xml:space="preserve">Automation Competitive Announcement </t>
-  </si>
-  <si>
     <t>Automation Formula Announcement</t>
   </si>
   <si>
@@ -214,6 +212,9 @@
   </si>
   <si>
     <t>Automation Competitive Announcement for pre-application</t>
+  </si>
+  <si>
+    <t>Automation Competitive Announcement</t>
   </si>
 </sst>
 </file>
@@ -649,6 +650,174 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -696,7 +865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -864,7 +1033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -901,7 +1070,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>200</v>
@@ -1025,7 +1194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1054,7 +1223,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1113,7 +1282,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1172,7 +1341,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1667,7 +1836,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>20</v>

</xml_diff>

<commit_message>
Merged PR 2849: Merge Deepika_prod to master
Created and Automated New Test Cases in Negotiations
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DACB11B-9C7B-4B63-AF0B-9C2BFD01EB67}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576A8C15-37AB-4F12-BC9D-C013C38BE69F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>

</xml_diff>

<commit_message>
Committing to checkout another branch
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576A8C15-37AB-4F12-BC9D-C013C38BE69F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2313DE-582D-491B-8CA3-A56E9080895D}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="6" activeTab="10" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -23,10 +23,11 @@
     <sheet name="Reviewer" sheetId="4" r:id="rId8"/>
     <sheet name="Creation Second Modal" sheetId="6" r:id="rId9"/>
     <sheet name="Creation Second Modal1" sheetId="14" r:id="rId10"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId11"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId12"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId13"/>
-    <sheet name="Sheet3" sheetId="13" r:id="rId14"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId11"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId12"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId13"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId14"/>
+    <sheet name="Sheet3" sheetId="13" r:id="rId15"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -818,6 +819,174 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -865,7 +1034,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1033,7 +1202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1194,7 +1363,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
created and updated test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2313DE-582D-491B-8CA3-A56E9080895D}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8535F329-3AE5-4B6C-B039-FD444D1E674F}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="6" activeTab="10" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="8" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -1739,7 +1739,7 @@
         <v>20</v>
       </c>
       <c r="C12">
-        <v>100000</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated site visits test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C091CAA-9870-4D56-901B-485B084481F0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295D0B85-D0DC-43B7-ACB6-C94E3087FD49}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -247,26 +247,46 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF00396B"/>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
       <name val="Helvetica"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDDDDDD"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDDDDDD"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -284,7 +304,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1719,7 +1741,7 @@
     <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1730,7 +1752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
added scenario and update progress report scenario
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22325"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0281DBE3-15CB-4490-BC3C-E53F70F6C052}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BE8F4D-A89B-4C2E-BE26-5239290E1243}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="9" activeTab="11" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -24,11 +24,12 @@
     <sheet name="Reviewer" sheetId="4" r:id="rId9"/>
     <sheet name="Creation Second Modal" sheetId="6" r:id="rId10"/>
     <sheet name="Creation Second Modal1" sheetId="14" r:id="rId11"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId12"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId13"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId14"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId15"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId16"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId12"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId13"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId14"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId15"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId16"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId17"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -594,14 +595,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -612,7 +613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -623,7 +624,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -634,7 +635,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -654,13 +655,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -671,7 +672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -682,7 +683,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -693,7 +694,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -704,7 +705,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -715,7 +716,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -726,7 +727,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -737,7 +738,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -748,7 +749,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -759,7 +760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -770,7 +771,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -781,7 +782,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -792,7 +793,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -803,7 +804,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -823,13 +824,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -840,7 +841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -851,7 +852,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -862,7 +863,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -873,7 +874,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -884,7 +885,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -895,7 +896,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -906,7 +907,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -917,7 +918,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -928,7 +929,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -939,7 +940,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -950,7 +951,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -961,7 +962,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -972,7 +973,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -989,15 +990,16 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1008,7 +1010,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1019,135 +1021,124 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1157,15 +1148,183 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1176,7 +1335,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1187,7 +1346,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1204,16 +1363,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1224,7 +1383,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1235,7 +1394,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1246,7 +1405,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1257,7 +1416,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1268,7 +1427,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1279,7 +1438,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1290,7 +1449,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1301,7 +1460,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1312,7 +1471,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1323,7 +1482,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1334,7 +1493,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1345,7 +1504,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1356,7 +1515,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1372,17 +1531,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1393,7 +1552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1404,7 +1563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1415,7 +1574,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1426,7 +1585,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1437,7 +1596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1448,7 +1607,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1459,7 +1618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1470,7 +1629,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1481,7 +1640,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1492,7 +1651,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1503,7 +1662,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1514,7 +1673,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1533,17 +1692,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1554,7 +1713,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1565,7 +1724,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1576,7 +1735,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1587,7 +1746,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1598,7 +1757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1609,7 +1768,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1620,7 +1779,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1631,7 +1790,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1642,7 +1801,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1653,7 +1812,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1664,7 +1823,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1675,7 +1834,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1686,7 +1845,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1705,14 +1864,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1723,7 +1882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1734,7 +1893,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1745,7 +1904,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1765,12 +1924,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1781,7 +1940,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1792,7 +1951,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1803,7 +1962,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1822,14 +1981,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1840,7 +1999,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1851,7 +2010,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1862,7 +2021,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1881,14 +2040,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1899,7 +2058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1910,7 +2069,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1921,7 +2080,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1941,14 +2100,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1959,7 +2118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1970,7 +2129,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1981,7 +2140,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1992,7 +2151,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2003,7 +2162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2014,7 +2173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2025,7 +2184,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2036,7 +2195,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2047,7 +2206,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2058,7 +2217,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2069,7 +2228,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2091,13 +2250,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2108,7 +2267,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2119,7 +2278,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2130,7 +2289,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2141,7 +2300,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2152,7 +2311,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2163,7 +2322,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2174,7 +2333,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2185,7 +2344,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2196,7 +2355,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2207,7 +2366,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2218,7 +2377,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2240,14 +2399,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2258,7 +2417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2269,7 +2428,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2288,13 +2447,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2305,7 +2464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2316,7 +2475,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2327,7 +2486,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2338,7 +2497,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2349,7 +2508,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
added new 5 scenarios
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BE8F4D-A89B-4C2E-BE26-5239290E1243}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19E03FF-2626-4025-A844-204D419C49A1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="9" activeTab="11" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="10" activeTab="12" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -25,11 +25,12 @@
     <sheet name="Creation Second Modal" sheetId="6" r:id="rId10"/>
     <sheet name="Creation Second Modal1" sheetId="14" r:id="rId11"/>
     <sheet name="Creation Second Modal3" sheetId="17" r:id="rId12"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId13"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId14"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId15"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId16"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId17"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId13"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId14"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId15"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId16"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId17"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId18"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="59">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -1148,6 +1149,164 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1315,7 +1474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1363,7 +1522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1531,7 +1690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1692,7 +1851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Added 5 test case and resolved issues
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19E03FF-2626-4025-A844-204D419C49A1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314E40B1-71D6-4AF6-BE3A-55901759D373}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="10" activeTab="12" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -1254,7 +1254,7 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
created new test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC84C94-AF19-4BAD-822D-53A3B3CA8EDB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3527BF50-E26E-4BA8-AE98-021F1B413466}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="12" activeTab="16" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="8" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -19,18 +19,20 @@
     <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId4"/>
     <sheet name="Creation" sheetId="7" r:id="rId5"/>
     <sheet name="Edition" sheetId="2" r:id="rId6"/>
-    <sheet name="Edition1" sheetId="10" r:id="rId7"/>
-    <sheet name="BudgetPeriod" sheetId="3" r:id="rId8"/>
-    <sheet name="Reviewer" sheetId="4" r:id="rId9"/>
-    <sheet name="Creation Second Modal" sheetId="6" r:id="rId10"/>
-    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId11"/>
-    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId12"/>
-    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId13"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId14"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId15"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId16"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId17"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId18"/>
+    <sheet name="AppDueDate" sheetId="20" r:id="rId7"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId8"/>
+    <sheet name="PreAppDueDate" sheetId="21" r:id="rId9"/>
+    <sheet name="BudgetPeriod" sheetId="3" r:id="rId10"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId11"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId12"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId13"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId14"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId15"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId16"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId17"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId18"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId19"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId20"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="62">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -122,9 +124,6 @@
     <t>QAContactEmailAddress__c</t>
   </si>
   <si>
-    <t>hema.ananthan@reisystems.com</t>
-  </si>
-  <si>
     <t>AwardFloor__c</t>
   </si>
   <si>
@@ -228,6 +227,9 @@
   </si>
   <si>
     <t>Automation</t>
+  </si>
+  <si>
+    <t>deepika.vanamala@reisystems.com</t>
   </si>
 </sst>
 </file>
@@ -631,7 +633,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -642,7 +644,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -663,6 +665,135 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3">
+        <v>379</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -734,7 +865,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -742,10 +873,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -753,7 +884,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -764,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -775,7 +906,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -786,7 +917,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -797,10 +928,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -808,10 +939,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -819,10 +950,10 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -831,7 +962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -911,10 +1042,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -922,7 +1053,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -933,7 +1064,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -944,7 +1075,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -955,7 +1086,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -966,10 +1097,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -977,10 +1108,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -988,10 +1119,10 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -999,7 +1130,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1069,10 +1200,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1080,7 +1211,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
@@ -1091,7 +1222,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1102,7 +1233,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1113,7 +1244,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1124,10 +1255,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1135,10 +1266,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1146,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1157,7 +1288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1227,10 +1358,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1238,7 +1369,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
@@ -1249,10 +1380,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1260,7 +1391,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1271,7 +1402,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1282,10 +1413,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1293,10 +1424,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1304,10 +1435,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1315,7 +1446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1395,10 +1526,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1406,10 +1537,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1417,7 +1548,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1428,7 +1559,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1439,7 +1570,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -1450,10 +1581,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1461,10 +1592,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1472,10 +1603,10 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1483,7 +1614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1508,10 +1639,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1519,10 +1650,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1531,7 +1662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1611,10 +1742,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1622,7 +1753,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1633,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1644,7 +1775,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1655,7 +1786,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -1666,10 +1797,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1677,10 +1808,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1688,10 +1819,10 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1699,7 +1830,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1725,183 +1856,14 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C9" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1937,7 +1899,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1948,7 +1910,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1965,6 +1927,175 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1996,7 +2127,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2007,7 +2138,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2055,7 +2186,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2066,7 +2197,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2114,7 +2245,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2125,7 +2256,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2185,7 +2316,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2240,7 +2371,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -2248,7 +2379,7 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9">
         <v>1000</v>
@@ -2270,7 +2401,7 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -2296,6 +2427,156 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>10000</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1" xr:uid="{D22297E3-ABE8-4F1A-B976-F74580C7D18E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2334,7 +2615,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2353,7 +2634,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5">
         <v>25</v>
@@ -2364,10 +2645,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2378,7 +2659,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2386,7 +2667,7 @@
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8">
         <v>1000</v>
@@ -2408,7 +2689,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -2431,14 +2712,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -2454,108 +2734,115 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2">
-        <v>20</v>
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
         <v>30</v>
       </c>
-      <c r="C3">
-        <v>379</v>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>100000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
created and AUtomaed New Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3527BF50-E26E-4BA8-AE98-021F1B413466}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DEADD05-8600-4DFF-A872-D502F1323F27}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="8" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="6" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="62">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -2428,7 +2428,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -2488,40 +2488,40 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>61</v>
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -2529,49 +2529,13 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C9">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10">
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12">
-        <v>10000</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C8" r:id="rId1" xr:uid="{D22297E3-ABE8-4F1A-B976-F74580C7D18E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
5TCAutomated35Yet And fixed failed TC
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,38 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13ACB185-8E42-47E2-BF6B-58B1A0647B42}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FCFF45-74E7-4326-BDF1-E8F22B579E29}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="5" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="2" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
     <sheet name="CompetitiveAnnouncement" sheetId="5" r:id="rId2"/>
-    <sheet name="CompetitiveAnnouncement1" sheetId="16" r:id="rId3"/>
-    <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId4"/>
-    <sheet name="Creation" sheetId="7" r:id="rId5"/>
-    <sheet name="Edition" sheetId="2" r:id="rId6"/>
-    <sheet name="AppDueDate" sheetId="20" r:id="rId7"/>
-    <sheet name="Edition1" sheetId="10" r:id="rId8"/>
-    <sheet name="PreAppDueDate" sheetId="21" r:id="rId9"/>
-    <sheet name="BudgetPeriod" sheetId="3" r:id="rId10"/>
-    <sheet name="Reviewer" sheetId="4" r:id="rId11"/>
-    <sheet name="Creation Second Modal" sheetId="6" r:id="rId12"/>
-    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId13"/>
-    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId14"/>
-    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId15"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId16"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId17"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId18"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId19"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId20"/>
+    <sheet name="CompetitivePastAnnouncement" sheetId="22" r:id="rId3"/>
+    <sheet name="CompetitiveAnnouncement1" sheetId="16" r:id="rId4"/>
+    <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId5"/>
+    <sheet name="Creation" sheetId="7" r:id="rId6"/>
+    <sheet name="Edition" sheetId="2" r:id="rId7"/>
+    <sheet name="AppDueDate" sheetId="20" r:id="rId8"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId9"/>
+    <sheet name="PreAppDueDate" sheetId="21" r:id="rId10"/>
+    <sheet name="BudgetPeriod" sheetId="3" r:id="rId11"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId12"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId13"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId14"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId15"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId16"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId17"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId18"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId19"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId20"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId21"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="63">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -230,6 +231,9 @@
   </si>
   <si>
     <t>Automation Competitive Announcement</t>
+  </si>
+  <si>
+    <t>Automation Competitive Past Announcement</t>
   </si>
 </sst>
 </file>
@@ -607,14 +611,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -625,7 +629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -636,7 +640,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -647,7 +651,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -665,16 +669,15 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -685,26 +688,114 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3">
-        <v>379</v>
+      <c r="C11">
+        <v>100000</v>
       </c>
     </row>
   </sheetData>
@@ -713,15 +804,63 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3">
+        <v>379</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -732,7 +871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -743,7 +882,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -754,7 +893,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -765,7 +904,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -776,7 +915,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -793,16 +932,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -813,7 +952,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -824,7 +963,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -835,7 +974,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -846,7 +985,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -857,7 +996,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -868,7 +1007,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -879,7 +1018,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -890,7 +1029,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -901,7 +1040,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -912,7 +1051,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -923,7 +1062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -934,7 +1073,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -945,7 +1084,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -962,16 +1101,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -982,7 +1121,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -993,7 +1132,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1004,7 +1143,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1015,7 +1154,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1026,7 +1165,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1037,7 +1176,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1048,7 +1187,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1059,7 +1198,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1070,7 +1209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1081,7 +1220,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1092,7 +1231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1103,7 +1242,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1114,7 +1253,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1122,164 +1261,6 @@
         <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1289,16 +1270,16 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1309,7 +1290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1320,7 +1301,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1331,7 +1312,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1342,7 +1323,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1353,7 +1334,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1364,7 +1345,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1375,7 +1356,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1383,10 +1364,10 @@
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1397,7 +1378,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1408,7 +1389,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1419,7 +1400,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1430,7 +1411,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1447,15 +1428,16 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1466,7 +1448,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1477,135 +1459,124 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1615,15 +1586,183 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1634,7 +1773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1645,7 +1784,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1662,16 +1801,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1682,7 +1821,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1693,7 +1832,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1704,7 +1843,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1715,7 +1854,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1726,7 +1865,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1737,7 +1876,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1748,7 +1887,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1759,7 +1898,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1770,7 +1909,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1781,7 +1920,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1792,7 +1931,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1803,7 +1942,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1814,7 +1953,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1824,46 +1963,6 @@
       <c r="C14" t="s">
         <v>36</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1873,14 +1972,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="59.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="59.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1891,7 +1990,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1902,7 +2001,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1913,7 +2012,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1931,16 +2030,56 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1951,7 +2090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1962,7 +2101,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1973,7 +2112,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1984,7 +2123,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1995,7 +2134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2006,7 +2145,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2017,7 +2156,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2028,7 +2167,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2039,7 +2178,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2050,7 +2189,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2061,7 +2200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2072,7 +2211,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2083,7 +2222,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2100,15 +2239,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="44.77734375" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2119,18 +2258,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2141,7 +2280,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2158,16 +2297,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2178,7 +2316,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2186,10 +2324,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2200,7 +2338,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2217,16 +2355,75 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2237,7 +2434,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2248,7 +2445,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2259,7 +2456,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2276,17 +2473,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2297,7 +2494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2308,7 +2505,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2319,7 +2516,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2330,7 +2527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2341,7 +2538,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2352,7 +2549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2363,7 +2560,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2374,7 +2571,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2385,7 +2582,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2396,7 +2593,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2407,7 +2604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2418,7 +2615,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G13">
         <v>0</v>
       </c>
@@ -2431,17 +2628,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2452,7 +2649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2463,7 +2660,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2474,7 +2671,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2485,7 +2682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2496,7 +2693,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -2507,7 +2704,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2518,7 +2715,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2529,7 +2726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2545,16 +2742,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2565,7 +2762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2576,7 +2773,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2587,7 +2784,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2598,7 +2795,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2609,7 +2806,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2620,7 +2817,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2631,7 +2828,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2642,7 +2839,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2653,7 +2850,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2664,7 +2861,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2679,139 +2876,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11">
-        <v>100000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
add new test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63CC65D3-D526-4DF1-8C52-53D404927ADC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DEB26B-9357-494A-905D-08CADB900039}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -615,14 +615,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -633,7 +633,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -644,7 +644,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -655,7 +655,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -675,13 +675,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +692,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -703,7 +703,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -714,7 +714,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -722,10 +722,10 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -733,10 +733,10 @@
         <v>56</v>
       </c>
       <c r="C5">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -747,7 +747,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -758,7 +758,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -769,7 +769,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -780,7 +780,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -791,7 +791,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -811,13 +811,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -828,7 +828,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -839,7 +839,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -850,7 +850,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -861,7 +861,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -872,7 +872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -883,7 +883,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -894,7 +894,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -905,7 +905,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -916,7 +916,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -927,7 +927,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -946,14 +946,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -964,7 +964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -975,7 +975,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -994,13 +994,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1075,13 +1075,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1180,7 +1180,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1191,7 +1191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1244,13 +1244,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1412,14 +1412,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1570,14 +1570,14 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1654,7 +1654,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1739,13 +1739,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1811,7 +1811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1877,7 +1877,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1907,13 +1907,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1955,14 +1955,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="59.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="59.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2015,13 +2015,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2183,14 +2183,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C9" s="3"/>
     </row>
   </sheetData>
@@ -2223,14 +2223,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2307,7 +2307,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2392,13 +2392,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{312DC3EE-E575-46F9-A9B5-EB471905BC17}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="65.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" customWidth="1"/>
+    <col min="3" max="3" width="65.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2450,13 +2450,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
-    <col min="3" max="3" width="46.5703125" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
+    <col min="3" max="3" width="46.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2467,7 +2467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2508,13 +2508,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="44.7109375" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2566,14 +2566,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2625,14 +2625,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2685,14 +2685,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2733,10 +2733,10 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2802,7 +2802,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G13">
         <v>0</v>
       </c>
@@ -2840,14 +2840,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2869,7 +2869,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2891,7 +2891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Added new Test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product_A\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A156CB91-B07C-4BB1-BE51-CB4A05B97EF8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D8F1F6-C812-440B-A98A-C648E961FA78}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="0" windowWidth="19190" windowHeight="10200" activeTab="1" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="10" yWindow="0" windowWidth="19190" windowHeight="10200" firstSheet="1" activeTab="3" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -247,7 +247,7 @@
     <t>Construction</t>
   </si>
   <si>
-    <t>Automation Competitiv Announcement for Application</t>
+    <t>Automation For Application Per announcement</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated announcement without ground feature file
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D5E412-0467-4159-A0C3-80140549F03F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2077C8E-946E-4C2C-9796-D8038F059207}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
@@ -3332,7 +3332,7 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated PreAppWB feature file
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2077C8E-946E-4C2C-9796-D8038F059207}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB282000-5FFF-431C-AE16-4A66C44D0532}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="5304" yWindow="1500" windowWidth="17280" windowHeight="8964" firstSheet="5" activeTab="6" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -220,9 +220,6 @@
     <t>PreApplicationDueDate__c</t>
   </si>
   <si>
-    <t>Automation Pre-App Announcement</t>
-  </si>
-  <si>
     <t>Justification__c</t>
   </si>
   <si>
@@ -235,9 +232,6 @@
     <t>Automation Competitive Past Announcement</t>
   </si>
   <si>
-    <t>Automation Announcement for Application Intake and PreApplication</t>
-  </si>
-  <si>
     <t>Construction</t>
   </si>
   <si>
@@ -251,6 +245,12 @@
   </si>
   <si>
     <t xml:space="preserve">Automation Runtime Directed Announcement </t>
+  </si>
+  <si>
+    <t>Automation Runtime Announcement for Pre-Application</t>
+  </si>
+  <si>
+    <t>Automation Runtime Announcement for Pre-App</t>
   </si>
 </sst>
 </file>
@@ -664,7 +664,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -793,7 +793,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2080,7 +2080,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2825,10 +2825,10 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" t="s">
         <v>57</v>
-      </c>
-      <c r="C2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -3037,7 +3037,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3100,7 +3100,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3157,8 +3157,8 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>61</v>
+      <c r="C2" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3185,6 +3185,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3216,7 +3217,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3273,8 +3274,8 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>56</v>
+      <c r="C2" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3301,6 +3302,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3333,7 +3335,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fixed announcement and application test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB282000-5FFF-431C-AE16-4A66C44D0532}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45333E3-697A-4E2F-86DC-2EA558FA1E0F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5304" yWindow="1500" windowWidth="17280" windowHeight="8964" firstSheet="5" activeTab="6" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="4097" yWindow="1029" windowWidth="16457" windowHeight="8554" firstSheet="6" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="66">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -229,28 +229,25 @@
     <t>deepika.vanamala@reisystems.com</t>
   </si>
   <si>
-    <t>Automation Competitive Past Announcement</t>
-  </si>
-  <si>
     <t>Construction</t>
   </si>
   <si>
-    <t>Automation For Application Per announcement</t>
-  </si>
-  <si>
     <t>Automation Runtime Formula Announcement</t>
   </si>
   <si>
     <t>Automation Runtime Competitive Announcement</t>
   </si>
   <si>
-    <t xml:space="preserve">Automation Runtime Directed Announcement </t>
-  </si>
-  <si>
     <t>Automation Runtime Announcement for Pre-Application</t>
   </si>
   <si>
     <t>Automation Runtime Announcement for Pre-App</t>
+  </si>
+  <si>
+    <t>Automation Runtime Directed Announcement</t>
+  </si>
+  <si>
+    <t>Automation Runtime Competitive Past Announcement</t>
   </si>
 </sst>
 </file>
@@ -638,14 +635,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.3046875" customWidth="1"/>
+    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -656,7 +653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -667,7 +664,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -678,7 +675,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -689,7 +686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="C12" s="5"/>
     </row>
   </sheetData>
@@ -701,14 +698,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -719,7 +716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -730,7 +727,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -741,7 +738,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -752,7 +749,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -763,7 +760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -774,7 +771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -785,7 +782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -796,7 +793,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -807,7 +804,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -818,7 +815,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -829,7 +826,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -840,7 +837,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="G13">
         <v>0</v>
       </c>
@@ -856,14 +853,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -874,7 +871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -885,7 +882,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -896,7 +893,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -907,7 +904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -918,7 +915,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -929,7 +926,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -940,7 +937,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -951,7 +948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -970,13 +967,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -987,7 +984,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -998,7 +995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1009,7 +1006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1020,7 +1017,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1031,7 +1028,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1042,7 +1039,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1053,7 +1050,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1064,7 +1061,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1075,7 +1072,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1086,7 +1083,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1106,13 +1103,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1123,7 +1120,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1134,7 +1131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1145,7 +1142,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1156,7 +1153,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1167,7 +1164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1178,7 +1175,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1189,7 +1186,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1200,7 +1197,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1211,7 +1208,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1222,7 +1219,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1241,14 +1238,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1259,7 +1256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1270,7 +1267,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1289,13 +1286,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1306,7 +1303,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1317,7 +1314,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1328,7 +1325,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1339,7 +1336,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1350,7 +1347,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1370,13 +1367,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1387,7 +1384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1398,7 +1395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1409,7 +1406,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1420,7 +1417,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1431,7 +1428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1442,7 +1439,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1453,7 +1450,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1464,7 +1461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1475,7 +1472,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1486,7 +1483,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1497,7 +1494,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1508,7 +1505,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1519,7 +1516,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1539,13 +1536,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1556,7 +1553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1567,7 +1564,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1578,7 +1575,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1589,7 +1586,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1600,7 +1597,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1611,7 +1608,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1622,7 +1619,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1633,7 +1630,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1644,7 +1641,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1655,7 +1652,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1666,7 +1663,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1677,7 +1674,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1696,13 +1693,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1713,7 +1710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1724,7 +1721,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1735,7 +1732,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1746,7 +1743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1757,7 +1754,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1768,7 +1765,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1779,7 +1776,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1790,7 +1787,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1801,7 +1798,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1812,7 +1809,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1823,7 +1820,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1834,7 +1831,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1845,7 +1842,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1864,13 +1861,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1881,7 +1878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1892,7 +1889,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1903,7 +1900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1914,7 +1911,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1925,7 +1922,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1936,7 +1933,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1947,7 +1944,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1958,7 +1955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1969,7 +1966,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1980,7 +1977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1991,7 +1988,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2002,7 +1999,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2013,7 +2010,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2032,14 +2029,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FC5EB7D-13BF-4B5E-895C-F5B651828B55}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
-    <col min="3" max="3" width="62.21875" customWidth="1"/>
+    <col min="1" max="1" width="30.4609375" customWidth="1"/>
+    <col min="2" max="2" width="26.3046875" customWidth="1"/>
+    <col min="3" max="3" width="62.23046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2050,7 +2047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2058,10 +2055,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2072,7 +2069,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2080,7 +2077,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2091,14 +2088,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.53515625" customWidth="1"/>
+    <col min="2" max="2" width="31.69140625" customWidth="1"/>
+    <col min="3" max="3" width="14.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,7 +2106,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2120,7 +2117,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2131,7 +2128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2142,7 +2139,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2153,7 +2150,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2164,7 +2161,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2175,7 +2172,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2186,7 +2183,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2197,7 +2194,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2208,7 +2205,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2219,7 +2216,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2230,7 +2227,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2249,14 +2246,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.53515625" customWidth="1"/>
+    <col min="2" max="2" width="24.4609375" customWidth="1"/>
+    <col min="3" max="3" width="15.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2267,7 +2264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2278,7 +2275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2289,7 +2286,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2300,7 +2297,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2311,7 +2308,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2322,7 +2319,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2333,7 +2330,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2344,7 +2341,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2355,7 +2352,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2366,7 +2363,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2377,7 +2374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2388,7 +2385,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2399,7 +2396,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2418,13 +2415,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2435,7 +2432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2446,7 +2443,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2457,7 +2454,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2468,7 +2465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2479,7 +2476,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2490,7 +2487,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2501,7 +2498,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2512,7 +2509,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2523,7 +2520,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2534,7 +2531,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2545,7 +2542,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2556,7 +2553,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2567,7 +2564,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2586,13 +2583,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2603,7 +2600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2614,7 +2611,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2634,13 +2631,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2651,7 +2648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2662,7 +2659,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2673,7 +2670,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2684,7 +2681,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2695,7 +2692,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2706,7 +2703,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2717,7 +2714,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2728,7 +2725,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2739,7 +2736,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2750,7 +2747,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2761,7 +2758,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2772,7 +2769,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2783,7 +2780,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2802,14 +2799,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2820,7 +2817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -2831,7 +2828,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="C9" s="3"/>
     </row>
   </sheetData>
@@ -2842,14 +2839,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.3046875" customWidth="1"/>
+    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2860,7 +2857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2871,7 +2868,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2882,7 +2879,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2893,7 +2890,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2904,7 +2901,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2915,7 +2912,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2926,7 +2923,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2937,7 +2934,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2948,7 +2945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2959,7 +2956,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2970,7 +2967,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2981,7 +2978,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2992,7 +2989,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -3011,14 +3008,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="59.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.3046875" customWidth="1"/>
+    <col min="3" max="3" width="59.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3029,7 +3026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3037,10 +3034,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3051,7 +3048,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3062,7 +3059,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="C9" s="5"/>
     </row>
   </sheetData>
@@ -3074,14 +3071,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801045D0-434D-4772-B50B-BAD32ADFCC6D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="1" max="1" width="33.84375" customWidth="1"/>
+    <col min="2" max="2" width="30.07421875" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3092,18 +3089,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3114,7 +3111,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3133,13 +3130,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{312DC3EE-E575-46F9-A9B5-EB471905BC17}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" customWidth="1"/>
-    <col min="3" max="3" width="65.88671875" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" customWidth="1"/>
+    <col min="3" max="3" width="65.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3150,7 +3147,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3158,10 +3155,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3172,7 +3169,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3192,13 +3189,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="31.33203125" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" customWidth="1"/>
+    <col min="2" max="2" width="31.3046875" customWidth="1"/>
+    <col min="3" max="3" width="46.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3209,7 +3206,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3217,10 +3214,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3231,7 +3228,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3250,13 +3247,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="44.6640625" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.69140625" customWidth="1"/>
+    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3267,7 +3264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3275,10 +3272,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3289,7 +3286,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3309,14 +3306,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.3046875" customWidth="1"/>
+    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3327,7 +3324,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3335,10 +3332,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3349,7 +3346,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3369,14 +3366,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.3046875" customWidth="1"/>
+    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3387,7 +3384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3398,7 +3395,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3409,7 +3406,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
updated Progress report, Amendment request, Auditor, Site visit, closeout
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45333E3-697A-4E2F-86DC-2EA558FA1E0F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED2AEB7-0F86-4252-80C7-9A5D80B137FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4097" yWindow="1029" windowWidth="16457" windowHeight="8554" firstSheet="6" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="10" activeTab="15" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="66">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -635,14 +635,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -653,7 +653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -664,7 +664,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -675,7 +675,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -686,7 +686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C12" s="5"/>
     </row>
   </sheetData>
@@ -698,14 +698,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.06640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -716,7 +716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -727,7 +727,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -738,7 +738,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -749,7 +749,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -760,7 +760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -771,7 +771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -782,7 +782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -793,7 +793,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -804,7 +804,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -815,7 +815,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -826,7 +826,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -837,7 +837,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="G13">
         <v>0</v>
       </c>
@@ -853,14 +853,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.06640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -871,7 +871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -882,7 +882,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -893,7 +893,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -915,7 +915,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -926,7 +926,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -937,7 +937,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -948,7 +948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -967,13 +967,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +984,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -995,7 +995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1103,13 +1103,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1238,14 +1238,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1286,13 +1286,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1366,14 +1366,14 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1439,91 +1439,80 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1536,13 +1525,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1542,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1564,7 +1553,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1575,7 +1564,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1586,7 +1575,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1597,7 +1586,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1608,7 +1597,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1619,7 +1608,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1630,7 +1619,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1641,7 +1630,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1652,7 +1641,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1663,7 +1652,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1674,7 +1663,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1693,13 +1682,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1710,7 +1699,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1721,7 +1710,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1732,7 +1721,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1743,7 +1732,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1754,7 +1743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1765,7 +1754,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1776,7 +1765,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1787,7 +1776,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1798,7 +1787,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1809,7 +1798,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1820,7 +1809,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1831,7 +1820,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1842,7 +1831,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1861,13 +1850,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1878,7 +1867,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1889,7 +1878,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1900,7 +1889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1911,7 +1900,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1922,7 +1911,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1933,7 +1922,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1944,7 +1933,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1955,7 +1944,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1966,7 +1955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1977,7 +1966,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1988,7 +1977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1999,7 +1988,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2010,7 +1999,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2029,14 +2018,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FC5EB7D-13BF-4B5E-895C-F5B651828B55}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="30.4609375" customWidth="1"/>
-    <col min="2" max="2" width="26.3046875" customWidth="1"/>
-    <col min="3" max="3" width="62.23046875" customWidth="1"/>
+    <col min="1" max="1" width="30.46484375" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="3" width="62.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2047,7 +2036,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2058,7 +2047,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2069,7 +2058,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2088,14 +2077,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.53515625" customWidth="1"/>
-    <col min="2" max="2" width="31.69140625" customWidth="1"/>
-    <col min="3" max="3" width="14.07421875" customWidth="1"/>
+    <col min="1" max="1" width="14.53125" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2106,7 +2095,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2117,7 +2106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2128,7 +2117,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2139,7 +2128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2150,7 +2139,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2161,7 +2150,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2172,7 +2161,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2183,7 +2172,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2194,7 +2183,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2205,7 +2194,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2216,7 +2205,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2227,7 +2216,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2246,14 +2235,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.53515625" customWidth="1"/>
-    <col min="2" max="2" width="24.4609375" customWidth="1"/>
-    <col min="3" max="3" width="15.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" customWidth="1"/>
+    <col min="2" max="2" width="24.46484375" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2253,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2275,7 +2264,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2286,7 +2275,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2297,7 +2286,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2308,7 +2297,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2319,7 +2308,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2330,7 +2319,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2341,7 +2330,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2352,7 +2341,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2363,7 +2352,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2374,7 +2363,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2385,7 +2374,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2396,7 +2385,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2415,13 +2404,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2432,7 +2421,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2443,7 +2432,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2454,7 +2443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2465,7 +2454,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2476,7 +2465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2487,7 +2476,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2498,7 +2487,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2509,7 +2498,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2520,7 +2509,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2531,7 +2520,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2542,7 +2531,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2553,7 +2542,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2564,7 +2553,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2583,13 +2572,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2600,7 +2589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2611,7 +2600,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2631,13 +2620,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2648,7 +2637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2659,7 +2648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2670,7 +2659,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2681,7 +2670,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2692,7 +2681,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2703,7 +2692,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2714,7 +2703,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2725,7 +2714,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2736,7 +2725,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2747,7 +2736,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2758,7 +2747,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2769,7 +2758,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2780,7 +2769,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -2799,14 +2788,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.06640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2817,7 +2806,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -2828,7 +2817,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C9" s="3"/>
     </row>
   </sheetData>
@@ -2839,14 +2828,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2857,7 +2846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2868,7 +2857,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2879,7 +2868,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2890,7 +2879,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2901,7 +2890,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2912,7 +2901,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2923,7 +2912,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2934,7 +2923,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2945,7 +2934,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2956,7 +2945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2967,7 +2956,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2978,7 +2967,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -2989,7 +2978,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -3008,14 +2997,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="59.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="59.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3026,7 +3015,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3037,7 +3026,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3048,7 +3037,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3059,7 +3048,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C9" s="5"/>
     </row>
   </sheetData>
@@ -3071,14 +3060,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801045D0-434D-4772-B50B-BAD32ADFCC6D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33.84375" customWidth="1"/>
-    <col min="2" max="2" width="30.07421875" customWidth="1"/>
+    <col min="1" max="1" width="33.86328125" customWidth="1"/>
+    <col min="2" max="2" width="30.06640625" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3089,7 +3078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3100,7 +3089,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3111,7 +3100,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3130,13 +3119,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{312DC3EE-E575-46F9-A9B5-EB471905BC17}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" customWidth="1"/>
-    <col min="3" max="3" width="65.84375" customWidth="1"/>
+    <col min="2" max="2" width="29.46484375" customWidth="1"/>
+    <col min="3" max="3" width="65.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3147,7 +3136,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3158,7 +3147,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3169,7 +3158,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3189,13 +3178,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="31.3046875" customWidth="1"/>
-    <col min="3" max="3" width="46.53515625" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
+    <col min="3" max="3" width="46.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3206,7 +3195,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3217,7 +3206,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3228,7 +3217,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3247,13 +3236,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="44.69140625" customWidth="1"/>
-    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3264,7 +3253,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3275,7 +3264,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3286,7 +3275,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3306,14 +3295,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3324,7 +3313,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3335,7 +3324,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3346,7 +3335,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3366,14 +3355,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3384,7 +3373,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3395,7 +3384,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3406,7 +3395,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Completed 14 test cases for RnR functionality with changes as per regression report/changes
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED2AEB7-0F86-4252-80C7-9A5D80B137FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BDB287A-FE8D-4989-930D-1F559DD37C6E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="10" activeTab="15" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="21" activeTab="23" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="66">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -1524,6 +1524,152 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1550,7 +1696,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1558,10 +1704,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
         <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1569,10 +1715,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -1580,10 +1726,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -1591,7 +1737,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1605,7 +1751,7 @@
         <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1616,7 +1762,7 @@
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -1627,7 +1773,7 @@
         <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -1679,9 +1825,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
-  <dimension ref="A1:C14"/>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
@@ -1751,7 +1897,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -1759,10 +1905,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1770,7 +1916,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1781,10 +1927,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -1792,7 +1938,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1803,10 +1949,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -1814,7 +1960,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -1825,188 +1971,9 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2076,7 +2043,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.53125" customWidth="1"/>
@@ -2144,10 +2111,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -2155,7 +2122,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
@@ -2166,7 +2133,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -2177,7 +2144,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -2188,10 +2155,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
@@ -2199,7 +2166,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -2210,20 +2177,9 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2234,7 +2190,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.53125" customWidth="1"/>
@@ -2313,10 +2269,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2324,10 +2280,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -2335,10 +2291,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -2346,7 +2302,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -2357,10 +2313,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -2368,7 +2324,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -2379,20 +2335,9 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2403,7 +2348,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
@@ -2481,10 +2426,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2492,10 +2437,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -2503,10 +2448,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -2514,7 +2459,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -2525,10 +2470,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -2536,7 +2481,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -2547,20 +2492,9 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2619,7 +2553,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
@@ -2697,10 +2631,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2708,7 +2642,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -2719,7 +2653,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -2730,7 +2664,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -2741,10 +2675,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -2752,7 +2686,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -2763,20 +2697,9 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated formula & directed modules
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8C8A1C-8344-4BED-9505-071DBB07905F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BF7017-CFFD-4E05-8425-1854BC91D963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="0" windowWidth="20355" windowHeight="10920" firstSheet="21" activeTab="21" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="75" yWindow="0" windowWidth="20355" windowHeight="10920" firstSheet="12" activeTab="13" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -281,9 +281,6 @@
     <t>fieldEligibleApplicantTypes__c</t>
   </si>
   <si>
-    <t>State governments;Individuals</t>
-  </si>
-  <si>
     <t>By Applicant and Focus Area</t>
   </si>
   <si>
@@ -297,6 +294,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>For Profit Organizations;Individuals</t>
   </si>
 </sst>
 </file>
@@ -986,7 +986,7 @@
         <v>15</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1103,7 +1103,7 @@
         <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1950,10 +1950,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2118,10 +2118,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2286,10 +2286,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -2456,10 +2456,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2625,10 +2625,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2940,10 +2940,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3108,10 +3108,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3266,10 +3266,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3435,10 +3435,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3661,10 +3661,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3877,10 +3877,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
done analysis for home module
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BF7017-CFFD-4E05-8425-1854BC91D963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E45CAF-60AE-49E4-BACC-E9D6366CA937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="75" yWindow="0" windowWidth="20355" windowHeight="10920" firstSheet="12" activeTab="13" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="45" yWindow="60" windowWidth="20355" windowHeight="10920" firstSheet="12" activeTab="13" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -1339,7 +1339,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1372,7 +1372,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -3181,7 +3181,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -3269,7 +3269,7 @@
         <v>71</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated for Application & Pre Application
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E45CAF-60AE-49E4-BACC-E9D6366CA937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{060F8AEE-4D86-46C9-9B00-C16ED0757874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="60" windowWidth="20355" windowHeight="10920" firstSheet="12" activeTab="13" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="135" yWindow="0" windowWidth="20355" windowHeight="10920" firstSheet="12" activeTab="14" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -1259,7 +1259,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3">

</xml_diff>

<commit_message>
update 1 test cases from 255648
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prod_Allocation_New_204\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B987936-84CD-4845-8DF2-DDD06ACAFDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E90DF4F6-2292-4695-AD5E-18D0A762BC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" firstSheet="26" activeTab="29" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" firstSheet="13" activeTab="15" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement_Admin" sheetId="44" r:id="rId1"/>
@@ -28,31 +28,32 @@
     <sheet name="CompetitivePastAnnouncement" sheetId="22" r:id="rId13"/>
     <sheet name="CompetitiveAnnouncement1" sheetId="16" r:id="rId14"/>
     <sheet name="FormulaAnn_AdminUser" sheetId="34" r:id="rId15"/>
-    <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId16"/>
-    <sheet name="Creation" sheetId="7" r:id="rId17"/>
-    <sheet name="Formula_Edition" sheetId="31" r:id="rId18"/>
-    <sheet name="Edition" sheetId="2" r:id="rId19"/>
-    <sheet name="AppDueDate" sheetId="20" r:id="rId20"/>
-    <sheet name="Edition1" sheetId="10" r:id="rId21"/>
-    <sheet name="PreAppDueDate" sheetId="21" r:id="rId22"/>
-    <sheet name="BudgetPeriod" sheetId="3" r:id="rId23"/>
-    <sheet name="Reviewer" sheetId="4" r:id="rId24"/>
-    <sheet name="Creation Second Negotiation" sheetId="29" r:id="rId25"/>
-    <sheet name="CreationFormula_ByApp_focusNo" sheetId="37" r:id="rId26"/>
-    <sheet name="Creation_Formula_ByApplicant" sheetId="35" r:id="rId27"/>
-    <sheet name="Creation_Formula_ByApp_FocusYes" sheetId="33" r:id="rId28"/>
-    <sheet name="Creation Second Modal" sheetId="6" r:id="rId29"/>
-    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId30"/>
-    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId31"/>
-    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId32"/>
-    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId33"/>
-    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId34"/>
-    <sheet name="Creation of pre-app_nego_yes" sheetId="15" r:id="rId35"/>
-    <sheet name="budget_Details_Subaward_Yes" sheetId="45" r:id="rId36"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId37"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId38"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId39"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId40"/>
+    <sheet name="FormulaAnn_AdminUser2" sheetId="46" r:id="rId16"/>
+    <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId17"/>
+    <sheet name="Creation" sheetId="7" r:id="rId18"/>
+    <sheet name="Formula_Edition" sheetId="31" r:id="rId19"/>
+    <sheet name="Edition" sheetId="2" r:id="rId20"/>
+    <sheet name="AppDueDate" sheetId="20" r:id="rId21"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId22"/>
+    <sheet name="PreAppDueDate" sheetId="21" r:id="rId23"/>
+    <sheet name="BudgetPeriod" sheetId="3" r:id="rId24"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId25"/>
+    <sheet name="Creation Second Negotiation" sheetId="29" r:id="rId26"/>
+    <sheet name="CreationFormula_ByApp_focusNo" sheetId="37" r:id="rId27"/>
+    <sheet name="Creation_Formula_ByApplicant" sheetId="35" r:id="rId28"/>
+    <sheet name="Creation_Formula_ByApp_FocusYes" sheetId="33" r:id="rId29"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId30"/>
+    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId31"/>
+    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId32"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId33"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId34"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId35"/>
+    <sheet name="Creation of pre-app_nego_yes" sheetId="15" r:id="rId36"/>
+    <sheet name="budget_Details_Subaward_Yes" sheetId="45" r:id="rId37"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId38"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId39"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId40"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId41"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="77">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -1150,6 +1151,64 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CB0B370-5042-41B9-A8EC-24D7CD1FD99D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="3" width="59.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <sheetPr codeName="Sheet15"/>
   <dimension ref="A1:C4"/>
@@ -1210,7 +1269,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:C4"/>
@@ -1271,7 +1330,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E513E26F-ED03-4E26-8F3C-BE6B3D3F87CC}">
   <sheetPr codeName="Sheet17"/>
   <dimension ref="A1:C9"/>
@@ -1386,163 +1445,6 @@
     <hyperlink ref="C8" r:id="rId1" xr:uid="{17978832-59AF-4679-BB70-8F18FAB7D619}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
-  <sheetPr codeName="Sheet18"/>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="G13">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C8" r:id="rId1" xr:uid="{F4D31CA5-8F43-42CF-8982-056FC1AEE3F1}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1607,6 +1509,163 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
+  <sheetPr codeName="Sheet18"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="G13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1" xr:uid="{F4D31CA5-8F43-42CF-8982-056FC1AEE3F1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:C9"/>
@@ -1721,7 +1780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <sheetPr codeName="Sheet20"/>
   <dimension ref="A1:C11"/>
@@ -1858,7 +1917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <sheetPr codeName="Sheet21"/>
   <dimension ref="A1:C11"/>
@@ -1994,7 +2053,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <sheetPr codeName="Sheet22"/>
   <dimension ref="A1:C3"/>
@@ -2043,7 +2102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <sheetPr codeName="Sheet23"/>
   <dimension ref="A1:C6"/>
@@ -2125,7 +2184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5689EA4D-03A7-4B71-84BE-6001E09A3DD3}">
   <sheetPr codeName="Sheet24"/>
   <dimension ref="A1:C14"/>
@@ -2295,7 +2354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366DB7B4-C63A-47E9-A3AB-3A17CFD5CE09}">
   <sheetPr codeName="Sheet25"/>
   <dimension ref="A1:C14"/>
@@ -2464,7 +2523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA6F82E-C68B-45AF-AB19-9A11877150E6}">
   <sheetPr codeName="Sheet26"/>
   <dimension ref="A1:C14"/>
@@ -2634,7 +2693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8CA48C-2A2F-44CF-A1AF-B3B67AA99C99}">
   <sheetPr codeName="Sheet27"/>
   <dimension ref="A1:C14"/>
@@ -2802,176 +2861,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
-  <sheetPr codeName="Sheet28"/>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3041,6 +2930,176 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
+  <sheetPr codeName="Sheet28"/>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <sheetPr codeName="Sheet29"/>
   <dimension ref="A1:C14"/>
@@ -3209,7 +3268,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <sheetPr codeName="Sheet30"/>
   <dimension ref="A1:C14"/>
@@ -3378,7 +3437,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:C14"/>
@@ -3547,7 +3606,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <sheetPr codeName="Sheet32"/>
   <dimension ref="A1:C13"/>
@@ -3706,7 +3765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <sheetPr codeName="Sheet33"/>
   <dimension ref="A1:C14"/>
@@ -3876,7 +3935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <sheetPr codeName="Sheet34"/>
   <dimension ref="A1:C14"/>
@@ -4045,7 +4104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B540E81-1FD2-4AA2-8DEE-8BFB8B274149}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4082,7 +4141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <sheetPr codeName="Sheet35"/>
   <dimension ref="A1:C3"/>
@@ -4131,7 +4190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <sheetPr codeName="Sheet36"/>
   <dimension ref="A1:C14"/>
@@ -4294,47 +4353,6 @@
       <c r="C14" s="7" t="s">
         <v>72</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
-  <sheetPr codeName="Sheet37"/>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4512,6 +4530,47 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
+  <sheetPr codeName="Sheet37"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="C9" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <sheetPr codeName="Sheet38"/>
   <dimension ref="A1:C14"/>

</xml_diff>

<commit_message>
Commit 2 test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\Product_Clone_Allocation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prod_Allocation_New_204\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3691D710-3771-4C16-91DF-00B045B74CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7ADA2B0-9448-4000-8A38-3B449A1B0D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" firstSheet="28" activeTab="29" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>

</xml_diff>

<commit_message>
Merged PR 13256: Merge vaibhav_allocation to Temp_Master_Allocation
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prod_Allocation_New_204\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\Product_Clone_Allocation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7ADA2B0-9448-4000-8A38-3B449A1B0D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E91A9C-548D-4FE6-80ED-7B1032D596D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" firstSheet="28" activeTab="29" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="795" firstSheet="16" activeTab="18" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement_Admin" sheetId="44" r:id="rId1"/>
@@ -840,7 +840,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1142,7 +1142,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1260,7 +1260,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1321,7 +1321,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -4968,7 +4968,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="62.140625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>